<commit_message>
Fix preview export coverage and gallery state restoration
Label and omit unresolved lookup relationships, include the Term Store asset, and restore captured site and interaction states from gallery links. Generate the full gallery license header and verify all links in fresh browser contexts. Regenerate the review artifacts and document the behavior.
</commit_message>
<xml_diff>
--- a/mockups/site-brief/review/sitenalyzer-synthetic-research-dictionary.xlsx
+++ b/mockups/site-brief/review/sitenalyzer-synthetic-research-dictionary.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">Export_Info!$A$1:$B$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">Sources!$A$1:$Q$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2">Assets!$A$1:$U$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2">Assets!$A$1:$U$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3">Fields!$A$1:$AH$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">Value_Sets!$A$1:$K$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5">Relationships!$A$1:$J$2</definedName>
@@ -647,7 +647,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U10"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -1257,10 +1257,75 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>00000000-0000-4000-8000-000000000001_termstore</v>
+      </c>
+      <c r="B10" t="str">
+        <v>00000000-0000-4000-8000-000000000001</v>
+      </c>
+      <c r="C10" t="str">
+        <v>TermStore</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Term Store</v>
+      </c>
+      <c r="E10" t="str">
+        <v>SharePoint Term Store</v>
+      </c>
+      <c r="F10" t="str">
+        <v>https://example.sharepoint.com/sites/research-example/_layouts/15/termstoremanager.aspx</v>
+      </c>
+      <c r="G10" t="str">
+        <v>https://example.sharepoint.com/sites/research-example</v>
+      </c>
+      <c r="H10" t="str">
+        <v>https://example.sharepoint.com/sites/research-example</v>
+      </c>
+      <c r="I10" t="str">
+        <v>SharePoint Managed Metadata term store</v>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v>Source</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Real-time</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="P10" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v>owner@example.org</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Active</v>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U9"/>
+  <autoFilter ref="A1:U10"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>